<commit_message>
Sharpen the SK Hynix piece: the leveraged-ETF rule change was dateable (28 Apr 2026)
Korea didn't just have looser leverage rules - it specifically banned
single-stock leveraged ETFs (10-stock minimum, 30% concentration cap)
until amending that rule on 28 April 2026, a month before the first
products launched. Added to both the write-up and the workbook
timeline; a real, dateable regulatory choice, not an inevitability.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/korea-leverage-crash-data.xlsx
+++ b/public/downloads/korea-leverage-crash-data.xlsx
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -685,153 +685,153 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Single-stock leveraged ETFs (2x daily) tied to Samsung and SK Hynix begin trading in Korea</t>
+          <t>Korea amends ETF rules, raising single-stock concentration limit from 30% to 100% (previously required 10+ stocks)</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Leverage</t>
+          <t>Policy</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>SK Hynix completes $26.5bn Nasdaq ADR listing — largest US listing ever by a foreign company</t>
+          <t>Single-stock leveraged ETFs (2x daily) tied to Samsung and SK Hynix begin trading in Korea</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Listing</t>
+          <t>Leverage</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Outstanding leveraged bets peak near W29.2tn (~$19.7bn); 1.2m retail accounts have hit margin calls</t>
+          <t>SK Hynix completes $26.5bn Nasdaq ADR listing — largest US listing ever by a foreign company</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Leverage</t>
+          <t>Listing</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Seoul-listed SK Hynix common shares fall 15.37%; the new Nasdaq ADR rises 27% the SAME day</t>
+          <t>Outstanding leveraged bets peak near W29.2tn (~$19.7bn); 1.2m retail accounts have hit margin calls</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>Leverage</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>KOSPI down ~25% from its June peak</t>
+          <t>Seoul-listed SK Hynix common shares fall 15.37%; the new Nasdaq ADR rises 27% the SAME day</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Index</t>
+          <t>Divergence</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Bank of Korea raises rates into an already-fragile market</t>
+          <t>KOSPI down ~25% from its June peak</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Macro</t>
+          <t>Index</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>China's Shanghai Aishengna reports mass production of homegrown immersion DUV lithography tools</t>
+          <t>Bank of Korea raises rates into an already-fragile market</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Competitive</t>
+          <t>Macro</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>SK Hynix reports Q2: revenue W79.32tn (+257% YoY), 76% operating margin — record quarter, missed ~W84tn consensus</t>
+          <t>China's Shanghai Aishengna reports mass production of homegrown immersion DUV lithography tools</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Earnings</t>
+          <t>Competitive</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Trough. SKHY ADR bottoms at $126.79. Government holds emergency market meeting after a 2-day W864.5tn wipeout</t>
+          <t>SK Hynix reports Q2: revenue W79.32tn (+257% YoY), 76% operating margin — record quarter, missed ~W84tn consensus</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Trough</t>
+          <t>Earnings</t>
         </is>
       </c>
     </row>
@@ -843,44 +843,61 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>FSC suspends new single-stock leveraged ETF listings, bans marketing, triples min. deposit to W30m</t>
+          <t>Trough. SKHY ADR bottoms at $126.79. Government holds emergency market meeting after a 2-day W864.5tn wipeout</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Policy</t>
+          <t>Trough</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>KOSPI +3.76% to 6,598 on US-Iran deal hopes</t>
+          <t>FSC suspends new single-stock leveraged ETF listings, bans marketing, triples min. deposit to W30m</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Rebound</t>
+          <t>Policy</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>KOSPI +3.76% to 6,598 on US-Iran deal hopes</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Rebound</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>KOSPI -4.58% to 6,296.38 as a broad Wall St. tech selloff hits Samsung (-6.5%) and SK Hynix (-10.67%)</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>Fresh selloff</t>
         </is>

</xml_diff>

<commit_message>
Fact-check SK Hynix piece and add native chart + sources to the Price Data sheet
Added the KOSPI's exact all-time-high level (9,385.59, 19 Jun), its record
+17.91% single-day surge on 31 July, and the specific SanDisk/Western Digital
guidance-miss trigger behind the 6 August selloff - all confirmed against
multiple independent sources and missing from the earlier draft. Also added
a native Excel line chart (SKHY vs. MU indexed, following the same dates as
the Timeline sheet) and a sources block directly under the Price Data sheet,
per request.
</commit_message>
<xml_diff>
--- a/public/downloads/korea-leverage-crash-data.xlsx
+++ b/public/downloads/korea-leverage-crash-data.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price Data" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leverage Data" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bull vs Bear" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Timeline" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Price Data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Leverage Data" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Bull vs Bear" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Sources" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,6 +70,11 @@
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00404040"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -132,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -153,6 +158,7 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -162,13 +168,13 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -243,6 +249,194 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SKHY (SK Hynix ADR) vs. MU (Micron), indexed to 100 on 2026-07-14</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Price Data'!C3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="BC5B33"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="4"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Price Data'!$A$4:$A$23</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Price Data'!$C$4:$C$23</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Price Data'!F3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="2F6F9F"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="4"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Price Data'!$A$4:$A$23</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Price Data'!$F$4:$F$23</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Indexed (7/14 = 100)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8640000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -650,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -719,68 +913,68 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>SK Hynix completes $26.5bn Nasdaq ADR listing — largest US listing ever by a foreign company</t>
+          <t>KOSPI closes at an all-time high of 9,385.59</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Listing</t>
+          <t>Index</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Outstanding leveraged bets peak near W29.2tn (~$19.7bn); 1.2m retail accounts have hit margin calls</t>
+          <t>SK Hynix completes $26.5bn Nasdaq ADR listing — largest US listing ever by a foreign company</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Leverage</t>
+          <t>Listing</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Seoul-listed SK Hynix common shares fall 15.37%; the new Nasdaq ADR rises 27% the SAME day</t>
+          <t>KOSPI down ~27% from its 19 June peak; outstanding leveraged bets peak near W29.2tn (~$19.7bn); 1.2m accounts hit margin calls</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Divergence</t>
+          <t>Leverage</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>KOSPI down ~25% from its June peak</t>
+          <t>Seoul-listed SK Hynix common shares fall 15.37%; the new Nasdaq ADR rises 27% the SAME day</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Index</t>
+          <t>Divergence</t>
         </is>
       </c>
     </row>
@@ -872,32 +1066,49 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>KOSPI +3.76% to 6,598 on US-Iran deal hopes</t>
+          <t>KOSPI +17.91% - largest single-day % and point gain in its history (prior record: 11.95%, Oct 2008). Samsung +28%, SK Hynix +30%</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Rebound</t>
+          <t>Record surge</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>KOSPI +3.76% to 6,598 on US-Iran deal hopes</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Rebound</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>KOSPI -4.58% to 6,296.38 as a broad Wall St. tech selloff hits Samsung (-6.5%) and SK Hynix (-10.67%)</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>KOSPI -4.58% to 6,296.38 - SanDisk/Western Digital beat estimates but missed on guidance, dragging SK Hynix (-9%) and Samsung (-6.3%) down in sympathy</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>Fresh selloff</t>
         </is>
@@ -914,7 +1125,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1582,8 +1793,65 @@
         <v/>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Chart follows the Timeline sheet's dates — see annotations there for what each move corresponds to.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="12" t="inlineStr">
+        <is>
+          <t>Sources for the price data on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>- SKHY and MU daily OHLCV — Twelve Data API (twelvedata.com), live-fetched 2026-08-07. Not a live feed: a dated snapshot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="14" t="inlineStr">
+        <is>
+          <t>- SK Hynix Seoul-listed shares -15.37% on 7/14 — Advisor Perspectives, https://www.advisorperspectives.com/articles/2026/07/13/sk-hynix-shares-plunge-record-deepening-korea-selloff</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>- KOSPI record +17.91% single-day gain, 7/31 — TradingKey, https://www.tradingkey.com/analysis/stocks/us-stocks/262067341-kospi-surged-17-9-percent-largest-single-day-gain-history-july-31-2026-tradingkey</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="14" t="inlineStr">
+        <is>
+          <t>- KOSPI all-time high 9,385.59 on 6/19 — IndMoney, https://www.indmoney.com/blog/us-stocks/kospi-index-crash-analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="14" t="inlineStr">
+        <is>
+          <t>- SanDisk/Western Digital guidance miss driving the 8/6 selloff — TradingKey, https://www.tradingkey.com/analysis/stocks/us-stocks/262082159-us-stock-sndk-wdc-skhy-mu-ai-tradingkey</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="14" t="inlineStr">
+        <is>
+          <t>- Samsung -6.3% close, SK Hynix selloff, 8/6 — Korea JoongAng Daily, https://www.koreajoongangdaily.com/business/kospi-slides-over-4-as-tech-shares-take-a-tumble/12812355</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1631,12 +1899,12 @@
           <t>Single-stock leveraged ETFs launched</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>27 May 2026</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>2x daily return products tied to Samsung / SK Hynix</t>
         </is>
@@ -1648,12 +1916,12 @@
           <t>Net retail purchases of leveraged ETFs</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>~W14tn (~$9.4bn)</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>vs. ~W2tn from foreign investors</t>
         </is>
@@ -1665,12 +1933,12 @@
           <t>Peak outstanding leveraged bets</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>W29.2tn (~$19.7bn)</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="16" t="inlineStr">
         <is>
           <t>Early July 2026</t>
         </is>
@@ -1682,12 +1950,12 @@
           <t>Retail accounts hitting margin calls</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>1,200,000+</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>As of 13 July 2026</t>
         </is>
@@ -1699,12 +1967,12 @@
           <t>Accounts forcibly liquidated</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>320,000 - 360,000</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>As of mid-July 2026</t>
         </is>
@@ -1716,12 +1984,12 @@
           <t>Total forced liquidation value</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>W2.3tn</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>Over ~2.5 months</t>
         </is>
@@ -1733,12 +2001,12 @@
           <t>New minimum deposit for leveraged investors (post-crisis)</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>W30m (~$20,000)</t>
         </is>
       </c>
-      <c r="C10" s="15" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>Tripled by the FSC, late July 2026</t>
         </is>
@@ -1750,12 +2018,12 @@
           <t>KOSPI single 2-day value wipeout</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>W864.5tn</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="C11" s="16" t="inlineStr">
         <is>
           <t>Triggered the 29 July emergency government meeting</t>
         </is>
@@ -1767,12 +2035,12 @@
           <t>President Lee Jae-myung disapproval rating</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>&gt;50%</t>
         </is>
       </c>
-      <c r="C12" s="15" t="inlineStr">
+      <c r="C12" s="16" t="inlineStr">
         <is>
           <t>First time in his term, per BigGo Finance / Bloombit reporting</t>
         </is>
@@ -1822,85 +2090,85 @@
       </c>
     </row>
     <row r="4" ht="70" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>SK Hynix Q2 result</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Revenue W79.32tn, +257% YoY, 76% operating margin — a genuine record quarter. 'Miss' vs. consensus (~W84tn) was a shipment-timing issue (HBM4 recognition slipping to Q3), not a demand problem.</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>Even a record quarter missed elevated Street expectations — a real sign the market had priced in near-perfection, leaving no room for anything less.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="70" customHeight="1">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Underlying AI demand</t>
         </is>
       </c>
-      <c r="B5" s="17" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>Hyperscaler 2026 capex guidance: Amazon $200bn, Alphabet $175-185bn, Meta $115-135bn, Microsoft $190bn — $725bn combined, +77% YoY. Evercore/BofA model &gt;$1tn combined for 2027. S&amp;P Global's July PMI showed the fastest tech-equipment output growth since May 2021.</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>Crowding and leverage across the whole AI trade (not just Korea) means positioning, not fundamentals, is doing a lot of the work in the price — a similar unwind could happen anywhere sentiment cracks next.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="70" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Analyst / investor commentary</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>J.P. Morgan (6 Aug note): the sell-off 'had not derailed' the AI investment cycle; 'we do not see any fundamental indicators that signal meaningful weakness in the next 6-12 months.'</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="C6" s="19" t="inlineStr">
         <is>
           <t>Michael Burry (4 Aug Substack): 'I continue to believe it is possible we are near a major top, and possibly a 1987-type fall.'</t>
         </is>
       </c>
     </row>
     <row r="7" ht="70" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>China competitive threat</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Currently immaterial in scale: ~5 domestic DUV units expected in 2026 vs. ASML's ~130 immersion systems; China's tools reportedly still lag ASML's technology.</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
+      <c r="C7" s="19" t="inlineStr">
         <is>
           <t>A real, credible first step toward Chinese self-sufficiency in a category it has never mass-produced before — a genuine multi-year strategic risk even if not a 2026-2027 supply/demand issue.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="70" customHeight="1">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>2027-2028 capacity</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>New capacity gives SK Hynix/Samsung/Micron room to keep growing into real, still-accelerating demand.</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
+      <c r="C8" s="19" t="inlineStr">
         <is>
           <t>Samsung, SK Hynix, Micron and Kioxia are all adding capacity simultaneously, due to reach volume in late 2027/2028 — right as hyperscaler capex growth may naturally decelerate off this year's exceptional base. The same setup that has ended every prior memory cycle.</t>
         </is>
@@ -1917,7 +2185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1958,7 +2226,7 @@
           <t>SK Hynix Nasdaq debut pricing — Bloomberg</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C4" s="20" t="inlineStr">
         <is>
           <t>https://www.bloomberg.com/news/articles/2026-07-09/sk-hynix-is-said-to-price-us-share-offering-at-149-apiece-mrdz562z</t>
         </is>
@@ -1973,7 +2241,7 @@
           <t>SK Hynix Nasdaq debut sets record — Yahoo Finance</t>
         </is>
       </c>
-      <c r="C5" s="19" t="inlineStr">
+      <c r="C5" s="20" t="inlineStr">
         <is>
           <t>https://finance.yahoo.com/markets/stocks/articles/sk-hynix-nasdaq-debut-26-113118390.html</t>
         </is>
@@ -1988,7 +2256,7 @@
           <t>Capital exodus hits KOSPI after ADR debut — Korea JoongAng Daily</t>
         </is>
       </c>
-      <c r="C6" s="19" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
         <is>
           <t>https://www.koreajoongangdaily.com/business/capital-exodus-hits-kospi-after-sk-hynixs-blockbuster-nasdaq-debut/12769678</t>
         </is>
@@ -2003,7 +2271,7 @@
           <t>Korean traders' leveraged bets unravel — CNBC</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
         <is>
           <t>https://www.cnbc.com/2026/07/20/give-me-my-money-back-south-korean-traders-leveraged-bets-unravel.html</t>
         </is>
@@ -2018,7 +2286,7 @@
           <t>Minister apologizes, leveraged ETF losses — CNBC</t>
         </is>
       </c>
-      <c r="C8" s="19" t="inlineStr">
+      <c r="C8" s="20" t="inlineStr">
         <is>
           <t>https://www.cnbc.com/2026/07/29/korea-leveraged-etf-kodex-sk-hynix.html</t>
         </is>
@@ -2033,7 +2301,7 @@
           <t>1.2 million accounts hit margin calls — BigGo Finance</t>
         </is>
       </c>
-      <c r="C9" s="19" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
         <is>
           <t>https://finance.biggo.com/news/1046f613-8e0d-4326-bd38-2d90a094e2cb</t>
         </is>
@@ -2048,7 +2316,7 @@
           <t>KOSPI plummets 23% in July, record circuit breakers — KuCoin</t>
         </is>
       </c>
-      <c r="C10" s="19" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>https://www.kucoin.com/news/flash/south-korea-s-kospi-index-plummets-23-in-july-2026-triggering-record-circuit-breakers</t>
         </is>
@@ -2063,7 +2331,7 @@
           <t>KOSPI crash worse than 1997 and 2008 — Yahoo Finance</t>
         </is>
       </c>
-      <c r="C11" s="19" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>https://finance.yahoo.com/markets/stocks/articles/south-korea-stock-market-crash-092957385.html</t>
         </is>
@@ -2078,7 +2346,7 @@
           <t>China begins mass-producing homegrown DUV tools — Tom's Hardware</t>
         </is>
       </c>
-      <c r="C12" s="19" t="inlineStr">
+      <c r="C12" s="20" t="inlineStr">
         <is>
           <t>https://www.tomshardware.com/tech-industry/semiconductors/china-begins-mass-production-of-domestic-immersion-duv-lithography-machines</t>
         </is>
@@ -2093,7 +2361,7 @@
           <t>China's chip breakthrough — the caveats — CNBC</t>
         </is>
       </c>
-      <c r="C13" s="19" t="inlineStr">
+      <c r="C13" s="20" t="inlineStr">
         <is>
           <t>https://www.cnbc.com/2026/07/28/china-chipmaking-duv-tool-asml-explained.html</t>
         </is>
@@ -2108,7 +2376,7 @@
           <t>SK hynix 2Q26 official results — SK hynix Newsroom</t>
         </is>
       </c>
-      <c r="C14" s="19" t="inlineStr">
+      <c r="C14" s="20" t="inlineStr">
         <is>
           <t>https://news.skhynix.com/en/q2-2026-business-results/</t>
         </is>
@@ -2123,7 +2391,7 @@
           <t>SK Hynix Q2 revenue +257% YoY — BigGo Finance</t>
         </is>
       </c>
-      <c r="C15" s="19" t="inlineStr">
+      <c r="C15" s="20" t="inlineStr">
         <is>
           <t>https://finance.biggo.com/news/KR_000660.KS_2026-07-28</t>
         </is>
@@ -2138,7 +2406,7 @@
           <t>Chip stocks shed $1tn in selloff — CNBC</t>
         </is>
       </c>
-      <c r="C16" s="19" t="inlineStr">
+      <c r="C16" s="20" t="inlineStr">
         <is>
           <t>https://www.cnbc.com/2026/07/29/chip-selloff-sk-hynix-samsung-softbank.html</t>
         </is>
@@ -2153,7 +2421,7 @@
           <t>Asian tech stocks drop, SK Hynix -10% — CNBC</t>
         </is>
       </c>
-      <c r="C17" s="19" t="inlineStr">
+      <c r="C17" s="20" t="inlineStr">
         <is>
           <t>https://www.cnbc.com/2026/08/06/asia-tech-selloff-wall-street-samsung-sk-hynix.html</t>
         </is>
@@ -2168,7 +2436,7 @@
           <t>Emergency meeting as W864tn leaves market — Yahoo Finance</t>
         </is>
       </c>
-      <c r="C18" s="19" t="inlineStr">
+      <c r="C18" s="20" t="inlineStr">
         <is>
           <t>https://finance.yahoo.com/markets/world-indices/articles/south-korea-holds-emergency-meeting-103240901.html</t>
         </is>
@@ -2183,7 +2451,7 @@
           <t>Kospi rout puts Lee government on alert — Bloomingbit</t>
         </is>
       </c>
-      <c r="C19" s="19" t="inlineStr">
+      <c r="C19" s="20" t="inlineStr">
         <is>
           <t>https://en.bloomingbit.io/feed/news/117526</t>
         </is>
@@ -2198,7 +2466,7 @@
           <t>NPS: an amplifier, not a stabilizer — Korea JoongAng Daily</t>
         </is>
       </c>
-      <c r="C20" s="19" t="inlineStr">
+      <c r="C20" s="20" t="inlineStr">
         <is>
           <t>https://www.koreajoongangdaily.com/opinion/nps-becomes-an-amplifier-not-a-stabilizer/12782277</t>
         </is>
@@ -2213,7 +2481,7 @@
           <t>KOSPI falls to 6,200 level, 6 August — Seoul Economic Daily</t>
         </is>
       </c>
-      <c r="C21" s="19" t="inlineStr">
+      <c r="C21" s="20" t="inlineStr">
         <is>
           <t>https://en.sedaily.com/finance/2026/08/06/kospi-falls-to-6200-level-as-chip-giants-plunge-kosdaq</t>
         </is>
@@ -2228,7 +2496,7 @@
           <t>Hyperscalers plan $725bn 2026 AI capex — AI Weekly</t>
         </is>
       </c>
-      <c r="C22" s="19" t="inlineStr">
+      <c r="C22" s="20" t="inlineStr">
         <is>
           <t>https://aiweekly.co/alerts/amazon-microsoft-alphabet-meta-plan-725b-ai-capex-in-2026</t>
         </is>
@@ -2243,7 +2511,7 @@
           <t>Michael Burry warns of 1987-type fall — CNBC</t>
         </is>
       </c>
-      <c r="C23" s="19" t="inlineStr">
+      <c r="C23" s="20" t="inlineStr">
         <is>
           <t>https://www.cnbc.com/2026/08/04/michael-burry-bets-against-rally-we-are-near-a-major-top.html</t>
         </is>
@@ -2258,7 +2526,7 @@
           <t>J.P. Morgan: AI investment cycle not derailed — CNBC</t>
         </is>
       </c>
-      <c r="C24" s="19" t="inlineStr">
+      <c r="C24" s="20" t="inlineStr">
         <is>
           <t>https://www.cnbc.com/2026/08/06/asia-tech-sell-off-has-not-derailed-ai-investment-cycle-jp-morgan-says.html</t>
         </is>
@@ -2273,9 +2541,69 @@
           <t>SKHY / MU daily price data — Twelve Data API</t>
         </is>
       </c>
-      <c r="C25" s="19" t="inlineStr">
+      <c r="C25" s="20" t="inlineStr">
         <is>
           <t>https://twelvedata.com (live-fetched 2026-08-07, see Price Data sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>KOSPI's record +17.91% single-day gain, 31 July — TradingKey</t>
+        </is>
+      </c>
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>https://www.tradingkey.com/analysis/stocks/us-stocks/262067341-kospi-surged-17-9-percent-largest-single-day-gain-history-july-31-2026-tradingkey</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>SanDisk/Western Digital guidance miss drags SK Hynix, Micron — TradingKey</t>
+        </is>
+      </c>
+      <c r="C27" s="20" t="inlineStr">
+        <is>
+          <t>https://www.tradingkey.com/analysis/stocks/us-stocks/262082159-us-stock-sndk-wdc-skhy-mu-ai-tradingkey</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>KOSPI all-time high of 9,385.59 on 19 June — IndMoney</t>
+        </is>
+      </c>
+      <c r="C28" s="20" t="inlineStr">
+        <is>
+          <t>https://www.indmoney.com/blog/us-stocks/kospi-index-crash-analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>KOSPI slides over 4% as tech shares tumble, 6 August — Korea JoongAng Daily</t>
+        </is>
+      </c>
+      <c r="C29" s="20" t="inlineStr">
+        <is>
+          <t>https://www.koreajoongangdaily.com/business/kospi-slides-over-4-as-tech-shares-take-a-tumble/12812355</t>
         </is>
       </c>
     </row>
@@ -2303,6 +2631,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cut the Read Me and Sources tabs, add explicit thesis rationale to Price Data
Removed the two workbook-navigation/index sheets since sources already live
at the end of the article - they were redundant. Added a stated "why MU,
why this matters" paragraph directly above the SKHY/MU summary numbers and
chart, explaining MU's role as the unlevered control group so the
comparison proves something rather than sitting there as two lines on a
chart.
</commit_message>
<xml_diff>
--- a/public/downloads/korea-leverage-crash-data.xlsx
+++ b/public/downloads/korea-leverage-crash-data.xlsx
@@ -7,12 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Timeline" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Price Data" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Leverage Data" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Bull vs Bear" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Sources" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Timeline" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Price Data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Leverage Data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Bull vs Bear" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,22 +38,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00595959"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00404040"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
@@ -67,9 +49,20 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -85,12 +78,6 @@
       <name val="Arial"/>
       <color rgb="00B71C1C"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="001155CC"/>
-      <sz val="9"/>
-      <u val="single"/>
     </font>
   </fonts>
   <fills count="4">
@@ -137,44 +124,44 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,7 +405,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>30</row>
+      <row>32</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3240000"/>
@@ -728,108 +715,273 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B17"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="2">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>Korea's Leverage Crash — Data Workbook</t>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Timeline — how the crash actually unfolded</t>
         </is>
       </c>
     </row>
     <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>SK Hynix, the KOSPI, and the July-August 2026 selloff — companion to the My Analysis write-up on bloombruh.com</t>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Korea amends ETF rules, raising single-stock concentration limit from 30% to 100% (previously required 10+ stocks)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Policy</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="3" t="inlineStr"/>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Single-stock leveraged ETFs (2x daily) tied to Samsung and SK Hynix begin trading in Korea</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Leverage</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>What's in this workbook:</t>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>KOSPI closes at an all-time high of 9,385.59</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Index</t>
         </is>
       </c>
     </row>
     <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Timeline        — the real, dated sequence of events, 10 July to 6 August 2026</t>
+          <t>SK Hynix completes $26.5bn Nasdaq ADR listing — largest US listing ever by a foreign company</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Listing</t>
         </is>
       </c>
     </row>
     <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Price Data      — real daily closes for SKHY (SK Hynix ADR) and MU (Micron), fetched live via Twelve Data,</t>
+          <t>KOSPI down ~27% from its 19 June peak; outstanding leveraged bets peak near W29.2tn (~$19.7bn); 1.2m accounts hit margin calls</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Leverage</t>
         </is>
       </c>
     </row>
     <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">                    plus indexed and daily % change columns (live formulas, not hardcoded)</t>
+          <t>Seoul-listed SK Hynix common shares fall 15.37%; the new Nasdaq ADR rises 27% the SAME day</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Divergence</t>
         </is>
       </c>
     </row>
     <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Leverage Data   — the leveraged-ETF and margin-call figures behind the crash's Korea-specific severity</t>
+          <t>Bank of Korea raises rates into an already-fragile market</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Macro</t>
         </is>
       </c>
     </row>
     <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Bull vs Bear    — the case for and against, in the same numbers used in the write-up</t>
+          <t>China's Shanghai Aishengna reports mass production of homegrown immersion DUV lithography tools</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Competitive</t>
         </is>
       </c>
     </row>
     <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Sources         — every source this workbook and the write-up draw on</t>
+          <t>SK Hynix reports Q2: revenue W79.32tn (+257% YoY), 76% operating margin — record quarter, missed ~W84tn consensus</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Earnings</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="3" t="inlineStr"/>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Trough. SKHY ADR bottoms at $126.79. Government holds emergency market meeting after a 2-day W864.5tn wipeout</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Trough</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Same discipline as every other model on this site: blue text is a hardcoded input (a real, sourced</t>
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>FSC suspends new single-stock leveraged ETF listings, bans marketing, triples min. deposit to W30m</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Policy</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>number), black text is a formula, yellow fill marks a figure worth double-checking against the live</t>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>KOSPI +17.91% - largest single-day % and point gain in its history (prior record: 11.95%, Oct 2008). Samsung +28%, SK Hynix +30%</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Record surge</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>chart on the site if you're using this for your own work. Nothing here is a live feed — every number</t>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>KOSPI +3.76% to 6,598 on US-Iran deal hopes</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Rebound</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>is a dated snapshot as of 7 August 2026.</t>
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>KOSPI -4.58% to 6,296.38 - SanDisk/Western Digital beat estimates but missed on guidance, dragging SK Hynix (-9%) and Samsung (-6.3%) down in sympathy</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Fresh selloff</t>
         </is>
       </c>
     </row>
@@ -844,288 +996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="95" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Timeline — how the crash actually unfolded</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Event</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Korea amends ETF rules, raising single-stock concentration limit from 30% to 100% (previously required 10+ stocks)</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Policy</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Single-stock leveraged ETFs (2x daily) tied to Samsung and SK Hynix begin trading in Korea</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Leverage</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-19</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>KOSPI closes at an all-time high of 9,385.59</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>Index</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>SK Hynix completes $26.5bn Nasdaq ADR listing — largest US listing ever by a foreign company</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Listing</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>KOSPI down ~27% from its 19 June peak; outstanding leveraged bets peak near W29.2tn (~$19.7bn); 1.2m accounts hit margin calls</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Leverage</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-14</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Seoul-listed SK Hynix common shares fall 15.37%; the new Nasdaq ADR rises 27% the SAME day</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Divergence</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Bank of Korea raises rates into an already-fragile market</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Macro</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>China's Shanghai Aishengna reports mass production of homegrown immersion DUV lithography tools</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Competitive</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>SK Hynix reports Q2: revenue W79.32tn (+257% YoY), 76% operating margin — record quarter, missed ~W84tn consensus</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>Earnings</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Trough. SKHY ADR bottoms at $126.79. Government holds emergency market meeting after a 2-day W864.5tn wipeout</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>Trough</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>FSC suspends new single-stock leveraged ETF listings, bans marketing, triples min. deposit to W30m</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Policy</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>KOSPI +17.91% - largest single-day % and point gain in its history (prior record: 11.95%, Oct 2008). Samsung +28%, SK Hynix +30%</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Record surge</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>KOSPI +3.76% to 6,598 on US-Iran deal hopes</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>Rebound</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>KOSPI -4.58% to 6,296.38 - SanDisk/Western Digital beat estimates but missed on guidance, dragging SK Hynix (-9%) and Samsung (-6.3%) down in sympathy</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>Fresh selloff</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1145,717 +1016,734 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>SKHY Close ($)</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>SKHY Indexed (7/14=100)</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>SKHY Daily % Chg</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>MU Close ($)</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>MU Indexed (7/14=100)</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>MU Daily % Chg</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="5" t="n">
         <v>168.01</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="6">
         <f>B4/$B$6*100</f>
         <v/>
       </c>
-      <c r="D4" s="10" t="n"/>
-      <c r="E4" s="8" t="n">
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="5" t="n">
         <v>979.3</v>
       </c>
-      <c r="F4" s="9">
+      <c r="F4" s="6">
         <f>E4/$E$6*100</f>
         <v/>
       </c>
-      <c r="G4" s="10" t="n"/>
+      <c r="G4" s="7" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="5" t="n">
         <v>152.35</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="6">
         <f>B5/$B$6*100</f>
         <v/>
       </c>
-      <c r="D5" s="11">
+      <c r="D5" s="8">
         <f>B5/B4-1</f>
         <v/>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="5" t="n">
         <v>937</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="6">
         <f>E5/$E$6*100</f>
         <v/>
       </c>
-      <c r="G5" s="11">
+      <c r="G5" s="8">
         <f>E5/E4-1</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="5" t="n">
         <v>193.92</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="6">
         <f>B6/$B$6*100</f>
         <v/>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="8">
         <f>B6/B5-1</f>
         <v/>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="5" t="n">
         <v>983.12</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F6" s="6">
         <f>E6/$E$6*100</f>
         <v/>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="8">
         <f>E6/E5-1</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="5" t="n">
         <v>176.46</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="6">
         <f>B7/$B$6*100</f>
         <v/>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="8">
         <f>B7/B6-1</f>
         <v/>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="5" t="n">
         <v>904.28</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="6">
         <f>E7/$E$6*100</f>
         <v/>
       </c>
-      <c r="G7" s="11">
+      <c r="G7" s="8">
         <f>E7/E6-1</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="5" t="n">
         <v>152.31</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C8" s="6">
         <f>B8/$B$6*100</f>
         <v/>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="8">
         <f>B8/B7-1</f>
         <v/>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="5" t="n">
         <v>853.2</v>
       </c>
-      <c r="F8" s="9">
+      <c r="F8" s="6">
         <f>E8/$E$6*100</f>
         <v/>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="8">
         <f>E8/E7-1</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="5" t="n">
         <v>154.03</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="6">
         <f>B9/$B$6*100</f>
         <v/>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="8">
         <f>B9/B8-1</f>
         <v/>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="5" t="n">
         <v>848.95</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="6">
         <f>E9/$E$6*100</f>
         <v/>
       </c>
-      <c r="G9" s="11">
+      <c r="G9" s="8">
         <f>E9/E8-1</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>2026-07-20</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="5" t="n">
         <v>151.16</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="6">
         <f>B10/$B$6*100</f>
         <v/>
       </c>
-      <c r="D10" s="11">
+      <c r="D10" s="8">
         <f>B10/B9-1</f>
         <v/>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="5" t="n">
         <v>865.46</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="6">
         <f>E10/$E$6*100</f>
         <v/>
       </c>
-      <c r="G10" s="11">
+      <c r="G10" s="8">
         <f>E10/E9-1</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>2026-07-21</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n">
+      <c r="B11" s="5" t="n">
         <v>171.94</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="6">
         <f>B11/$B$6*100</f>
         <v/>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="8">
         <f>B11/B10-1</f>
         <v/>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="5" t="n">
         <v>970.8200000000001</v>
       </c>
-      <c r="F11" s="9">
+      <c r="F11" s="6">
         <f>E11/$E$6*100</f>
         <v/>
       </c>
-      <c r="G11" s="11">
+      <c r="G11" s="8">
         <f>E11/E10-1</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>2026-07-22</t>
         </is>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B12" s="5" t="n">
         <v>165.27</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="6">
         <f>B12/$B$6*100</f>
         <v/>
       </c>
-      <c r="D12" s="11">
+      <c r="D12" s="8">
         <f>B12/B11-1</f>
         <v/>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="E12" s="5" t="n">
         <v>959.48</v>
       </c>
-      <c r="F12" s="9">
+      <c r="F12" s="6">
         <f>E12/$E$6*100</f>
         <v/>
       </c>
-      <c r="G12" s="11">
+      <c r="G12" s="8">
         <f>E12/E11-1</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="5" t="n">
         <v>169.5</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="6">
         <f>B13/$B$6*100</f>
         <v/>
       </c>
-      <c r="D13" s="11">
+      <c r="D13" s="8">
         <f>B13/B12-1</f>
         <v/>
       </c>
-      <c r="E13" s="8" t="n">
+      <c r="E13" s="5" t="n">
         <v>990.21</v>
       </c>
-      <c r="F13" s="9">
+      <c r="F13" s="6">
         <f>E13/$E$6*100</f>
         <v/>
       </c>
-      <c r="G13" s="11">
+      <c r="G13" s="8">
         <f>E13/E12-1</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>2026-07-24</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="5" t="n">
         <v>154.57</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="6">
         <f>B14/$B$6*100</f>
         <v/>
       </c>
-      <c r="D14" s="11">
+      <c r="D14" s="8">
         <f>B14/B13-1</f>
         <v/>
       </c>
-      <c r="E14" s="8" t="n">
+      <c r="E14" s="5" t="n">
         <v>920.95</v>
       </c>
-      <c r="F14" s="9">
+      <c r="F14" s="6">
         <f>E14/$E$6*100</f>
         <v/>
       </c>
-      <c r="G14" s="11">
+      <c r="G14" s="8">
         <f>E14/E13-1</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="B15" s="8" t="n">
+      <c r="B15" s="5" t="n">
         <v>143.02</v>
       </c>
-      <c r="C15" s="9">
+      <c r="C15" s="6">
         <f>B15/$B$6*100</f>
         <v/>
       </c>
-      <c r="D15" s="11">
+      <c r="D15" s="8">
         <f>B15/B14-1</f>
         <v/>
       </c>
-      <c r="E15" s="8" t="n">
+      <c r="E15" s="5" t="n">
         <v>900.2</v>
       </c>
-      <c r="F15" s="9">
+      <c r="F15" s="6">
         <f>E15/$E$6*100</f>
         <v/>
       </c>
-      <c r="G15" s="11">
+      <c r="G15" s="8">
         <f>E15/E14-1</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="B16" s="8" t="n">
+      <c r="B16" s="5" t="n">
         <v>130.17</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="6">
         <f>B16/$B$6*100</f>
         <v/>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="8">
         <f>B16/B15-1</f>
         <v/>
       </c>
-      <c r="E16" s="8" t="n">
+      <c r="E16" s="5" t="n">
         <v>820.53</v>
       </c>
-      <c r="F16" s="9">
+      <c r="F16" s="6">
         <f>E16/$E$6*100</f>
         <v/>
       </c>
-      <c r="G16" s="11">
+      <c r="G16" s="8">
         <f>E16/E15-1</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="B17" s="8" t="n">
+      <c r="B17" s="5" t="n">
         <v>126.79</v>
       </c>
-      <c r="C17" s="9">
+      <c r="C17" s="6">
         <f>B17/$B$6*100</f>
         <v/>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="8">
         <f>B17/B16-1</f>
         <v/>
       </c>
-      <c r="E17" s="8" t="n">
+      <c r="E17" s="5" t="n">
         <v>739</v>
       </c>
-      <c r="F17" s="9">
+      <c r="F17" s="6">
         <f>E17/$E$6*100</f>
         <v/>
       </c>
-      <c r="G17" s="11">
+      <c r="G17" s="8">
         <f>E17/E16-1</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="B18" s="8" t="n">
+      <c r="B18" s="5" t="n">
         <v>149</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="6">
         <f>B18/$B$6*100</f>
         <v/>
       </c>
-      <c r="D18" s="11">
+      <c r="D18" s="8">
         <f>B18/B17-1</f>
         <v/>
       </c>
-      <c r="E18" s="8" t="n">
+      <c r="E18" s="5" t="n">
         <v>874.66</v>
       </c>
-      <c r="F18" s="9">
+      <c r="F18" s="6">
         <f>E18/$E$6*100</f>
         <v/>
       </c>
-      <c r="G18" s="11">
+      <c r="G18" s="8">
         <f>E18/E17-1</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="B19" s="8" t="n">
+      <c r="B19" s="5" t="n">
         <v>143.73</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="6">
         <f>B19/$B$6*100</f>
         <v/>
       </c>
-      <c r="D19" s="11">
+      <c r="D19" s="8">
         <f>B19/B18-1</f>
         <v/>
       </c>
-      <c r="E19" s="8" t="n">
+      <c r="E19" s="5" t="n">
         <v>823.03</v>
       </c>
-      <c r="F19" s="9">
+      <c r="F19" s="6">
         <f>E19/$E$6*100</f>
         <v/>
       </c>
-      <c r="G19" s="11">
+      <c r="G19" s="8">
         <f>E19/E18-1</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="B20" s="8" t="n">
+      <c r="B20" s="5" t="n">
         <v>142.72</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="6">
         <f>B20/$B$6*100</f>
         <v/>
       </c>
-      <c r="D20" s="11">
+      <c r="D20" s="8">
         <f>B20/B19-1</f>
         <v/>
       </c>
-      <c r="E20" s="8" t="n">
+      <c r="E20" s="5" t="n">
         <v>829.5</v>
       </c>
-      <c r="F20" s="9">
+      <c r="F20" s="6">
         <f>E20/$E$6*100</f>
         <v/>
       </c>
-      <c r="G20" s="11">
+      <c r="G20" s="8">
         <f>E20/E19-1</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="B21" s="8" t="n">
+      <c r="B21" s="5" t="n">
         <v>154.38</v>
       </c>
-      <c r="C21" s="9">
+      <c r="C21" s="6">
         <f>B21/$B$6*100</f>
         <v/>
       </c>
-      <c r="D21" s="11">
+      <c r="D21" s="8">
         <f>B21/B20-1</f>
         <v/>
       </c>
-      <c r="E21" s="8" t="n">
+      <c r="E21" s="5" t="n">
         <v>892.67</v>
       </c>
-      <c r="F21" s="9">
+      <c r="F21" s="6">
         <f>E21/$E$6*100</f>
         <v/>
       </c>
-      <c r="G21" s="11">
+      <c r="G21" s="8">
         <f>E21/E20-1</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="B22" s="8" t="n">
+      <c r="B22" s="5" t="n">
         <v>151.03</v>
       </c>
-      <c r="C22" s="9">
+      <c r="C22" s="6">
         <f>B22/$B$6*100</f>
         <v/>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="8">
         <f>B22/B21-1</f>
         <v/>
       </c>
-      <c r="E22" s="8" t="n">
+      <c r="E22" s="5" t="n">
         <v>893.1900000000001</v>
       </c>
-      <c r="F22" s="9">
+      <c r="F22" s="6">
         <f>E22/$E$6*100</f>
         <v/>
       </c>
-      <c r="G22" s="11">
+      <c r="G22" s="8">
         <f>E22/E21-1</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="B23" s="8" t="n">
+      <c r="B23" s="5" t="n">
         <v>145.87</v>
       </c>
-      <c r="C23" s="9">
+      <c r="C23" s="6">
         <f>B23/$B$6*100</f>
         <v/>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="8">
         <f>B23/B22-1</f>
         <v/>
       </c>
-      <c r="E23" s="8" t="n">
+      <c r="E23" s="5" t="n">
         <v>898.97</v>
       </c>
-      <c r="F23" s="9">
+      <c r="F23" s="6">
         <f>E23/$E$6*100</f>
         <v/>
       </c>
-      <c r="G23" s="11">
+      <c r="G23" s="8">
         <f>E23/E22-1</f>
         <v/>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="12" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>Why MU, and why this matters for the thesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="105" customHeight="1">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>MU (Micron) is the control group. It's a comparable, US-listed memory-chip maker riding the exact same global AI/memory demand cycle as SK Hynix — but with zero exposure to Korea's leveraged-ETF machinery, margin calls, or forced retail liquidations, because it isn't a Korean stock. If Korea-specific leverage were the main driver of SK Hynix's crash, MU should have barely moved over the same window. It didn't: MU fell 24.8% while SKHY fell 34.6% — nearly as much, on a stock with none of Korea's leverage mechanics attached to it. That's the evidence for the article's central claim: most of SK Hynix's drawdown is the same global correction that hit an unlevered peer almost as hard. Korea's leverage machinery accounts for the incremental ~10 points below (see 'Implied Korea-specific incremental damage') and for nearly all of the margin-call/social fallout — not for the bulk of the price move itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>Peak (7/14) to trough (7/29):</t>
         </is>
       </c>
-      <c r="B26" s="12" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>SKHY drawdown</t>
         </is>
       </c>
-      <c r="C26" s="13">
+      <c r="C28" s="11">
         <f>B17/B6-1</f>
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="12" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>MU drawdown (unlevered US peer, same window)</t>
         </is>
       </c>
-      <c r="C27" s="13">
+      <c r="C29" s="11">
         <f>E17/E6-1</f>
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="12" t="inlineStr">
+    <row r="30">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Implied 'Korea-specific' incremental damage</t>
         </is>
       </c>
-      <c r="C28" s="13">
-        <f>C26-C27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="C30" s="11">
+        <f>C28-C29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
         <is>
           <t>Chart follows the Timeline sheet's dates — see annotations there for what each move corresponds to.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="12" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr">
         <is>
           <t>Sources for the price data on this sheet</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="14" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="13" t="inlineStr">
         <is>
           <t>- SKHY and MU daily OHLCV — Twelve Data API (twelvedata.com), live-fetched 2026-08-07. Not a live feed: a dated snapshot.</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="14" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="13" t="inlineStr">
         <is>
           <t>- SK Hynix Seoul-listed shares -15.37% on 7/14 — Advisor Perspectives, https://www.advisorperspectives.com/articles/2026/07/13/sk-hynix-shares-plunge-record-deepening-korea-selloff</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="14" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="13" t="inlineStr">
         <is>
           <t>- KOSPI record +17.91% single-day gain, 7/31 — TradingKey, https://www.tradingkey.com/analysis/stocks/us-stocks/262067341-kospi-surged-17-9-percent-largest-single-day-gain-history-july-31-2026-tradingkey</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="14" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="13" t="inlineStr">
         <is>
           <t>- KOSPI all-time high 9,385.59 on 6/19 — IndMoney, https://www.indmoney.com/blog/us-stocks/kospi-index-crash-analysis</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="14" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="13" t="inlineStr">
         <is>
           <t>- SanDisk/Western Digital guidance miss driving the 8/6 selloff — TradingKey, https://www.tradingkey.com/analysis/stocks/us-stocks/262082159-us-stock-sndk-wdc-skhy-mu-ai-tradingkey</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="14" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="13" t="inlineStr">
         <is>
           <t>- Samsung -6.3% close, SK Hynix selloff, 8/6 — Korea JoongAng Daily, https://www.koreajoongangdaily.com/business/kospi-slides-over-4-as-tech-shares-take-a-tumble/12812355</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A26:G26"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1877,170 +1765,170 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Figure</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Source / note</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Single-stock leveraged ETFs launched</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>27 May 2026</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>2x daily return products tied to Samsung / SK Hynix</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Net retail purchases of leveraged ETFs</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>~W14tn (~$9.4bn)</t>
         </is>
       </c>
-      <c r="C5" s="16" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>vs. ~W2tn from foreign investors</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Peak outstanding leveraged bets</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>W29.2tn (~$19.7bn)</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Early July 2026</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Retail accounts hitting margin calls</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>1,200,000+</t>
         </is>
       </c>
-      <c r="C7" s="16" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>As of 13 July 2026</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Accounts forcibly liquidated</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>320,000 - 360,000</t>
         </is>
       </c>
-      <c r="C8" s="16" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>As of mid-July 2026</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Total forced liquidation value</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>W2.3tn</t>
         </is>
       </c>
-      <c r="C9" s="16" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>Over ~2.5 months</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>New minimum deposit for leveraged investors (post-crisis)</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>W30m (~$20,000)</t>
         </is>
       </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <t>Tripled by the FSC, late July 2026</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>KOSPI single 2-day value wipeout</t>
         </is>
       </c>
-      <c r="B11" s="15" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>W864.5tn</t>
         </is>
       </c>
-      <c r="C11" s="16" t="inlineStr">
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <t>Triggered the 29 July emergency government meeting</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>President Lee Jae-myung disapproval rating</t>
         </is>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>&gt;50%</t>
         </is>
       </c>
-      <c r="C12" s="16" t="inlineStr">
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <t>First time in his term, per BigGo Finance / Bloombit reporting</t>
         </is>
@@ -2051,7 +1939,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2073,102 +1961,102 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Theme</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Bull case</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Bear case</t>
         </is>
       </c>
     </row>
     <row r="4" ht="70" customHeight="1">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>SK Hynix Q2 result</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>Revenue W79.32tn, +257% YoY, 76% operating margin — a genuine record quarter. 'Miss' vs. consensus (~W84tn) was a shipment-timing issue (HBM4 recognition slipping to Q3), not a demand problem.</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Even a record quarter missed elevated Street expectations — a real sign the market had priced in near-perfection, leaving no room for anything less.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="70" customHeight="1">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Underlying AI demand</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Hyperscaler 2026 capex guidance: Amazon $200bn, Alphabet $175-185bn, Meta $115-135bn, Microsoft $190bn — $725bn combined, +77% YoY. Evercore/BofA model &gt;$1tn combined for 2027. S&amp;P Global's July PMI showed the fastest tech-equipment output growth since May 2021.</t>
         </is>
       </c>
-      <c r="C5" s="19" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>Crowding and leverage across the whole AI trade (not just Korea) means positioning, not fundamentals, is doing a lot of the work in the price — a similar unwind could happen anywhere sentiment cracks next.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="70" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>Analyst / investor commentary</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>J.P. Morgan (6 Aug note): the sell-off 'had not derailed' the AI investment cycle; 'we do not see any fundamental indicators that signal meaningful weakness in the next 6-12 months.'</t>
         </is>
       </c>
-      <c r="C6" s="19" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>Michael Burry (4 Aug Substack): 'I continue to believe it is possible we are near a major top, and possibly a 1987-type fall.'</t>
         </is>
       </c>
     </row>
     <row r="7" ht="70" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>China competitive threat</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Currently immaterial in scale: ~5 domestic DUV units expected in 2026 vs. ASML's ~130 immersion systems; China's tools reportedly still lag ASML's technology.</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>A real, credible first step toward Chinese self-sufficiency in a category it has never mass-produced before — a genuine multi-year strategic risk even if not a 2026-2027 supply/demand issue.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="70" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>2027-2028 capacity</t>
         </is>
       </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>New capacity gives SK Hynix/Samsung/Micron room to keep growing into real, still-accelerating demand.</t>
         </is>
       </c>
-      <c r="C8" s="19" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>Samsung, SK Hynix, Micron and Kioxia are all adding capacity simultaneously, due to reach volume in late 2027/2028 — right as hyperscaler capex growth may naturally decelerate off this year's exceptional base. The same setup that has ended every prior memory cycle.</t>
         </is>
@@ -2177,465 +2065,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Sources</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>SK Hynix Nasdaq debut pricing — Bloomberg</t>
-        </is>
-      </c>
-      <c r="C4" s="20" t="inlineStr">
-        <is>
-          <t>https://www.bloomberg.com/news/articles/2026-07-09/sk-hynix-is-said-to-price-us-share-offering-at-149-apiece-mrdz562z</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>SK Hynix Nasdaq debut sets record — Yahoo Finance</t>
-        </is>
-      </c>
-      <c r="C5" s="20" t="inlineStr">
-        <is>
-          <t>https://finance.yahoo.com/markets/stocks/articles/sk-hynix-nasdaq-debut-26-113118390.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Capital exodus hits KOSPI after ADR debut — Korea JoongAng Daily</t>
-        </is>
-      </c>
-      <c r="C6" s="20" t="inlineStr">
-        <is>
-          <t>https://www.koreajoongangdaily.com/business/capital-exodus-hits-kospi-after-sk-hynixs-blockbuster-nasdaq-debut/12769678</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>Korean traders' leveraged bets unravel — CNBC</t>
-        </is>
-      </c>
-      <c r="C7" s="20" t="inlineStr">
-        <is>
-          <t>https://www.cnbc.com/2026/07/20/give-me-my-money-back-south-korean-traders-leveraged-bets-unravel.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>Minister apologizes, leveraged ETF losses — CNBC</t>
-        </is>
-      </c>
-      <c r="C8" s="20" t="inlineStr">
-        <is>
-          <t>https://www.cnbc.com/2026/07/29/korea-leveraged-etf-kodex-sk-hynix.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>1.2 million accounts hit margin calls — BigGo Finance</t>
-        </is>
-      </c>
-      <c r="C9" s="20" t="inlineStr">
-        <is>
-          <t>https://finance.biggo.com/news/1046f613-8e0d-4326-bd38-2d90a094e2cb</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>KOSPI plummets 23% in July, record circuit breakers — KuCoin</t>
-        </is>
-      </c>
-      <c r="C10" s="20" t="inlineStr">
-        <is>
-          <t>https://www.kucoin.com/news/flash/south-korea-s-kospi-index-plummets-23-in-july-2026-triggering-record-circuit-breakers</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>KOSPI crash worse than 1997 and 2008 — Yahoo Finance</t>
-        </is>
-      </c>
-      <c r="C11" s="20" t="inlineStr">
-        <is>
-          <t>https://finance.yahoo.com/markets/stocks/articles/south-korea-stock-market-crash-092957385.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>China begins mass-producing homegrown DUV tools — Tom's Hardware</t>
-        </is>
-      </c>
-      <c r="C12" s="20" t="inlineStr">
-        <is>
-          <t>https://www.tomshardware.com/tech-industry/semiconductors/china-begins-mass-production-of-domestic-immersion-duv-lithography-machines</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>China's chip breakthrough — the caveats — CNBC</t>
-        </is>
-      </c>
-      <c r="C13" s="20" t="inlineStr">
-        <is>
-          <t>https://www.cnbc.com/2026/07/28/china-chipmaking-duv-tool-asml-explained.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="n">
-        <v>11</v>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>SK hynix 2Q26 official results — SK hynix Newsroom</t>
-        </is>
-      </c>
-      <c r="C14" s="20" t="inlineStr">
-        <is>
-          <t>https://news.skhynix.com/en/q2-2026-business-results/</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="n">
-        <v>12</v>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>SK Hynix Q2 revenue +257% YoY — BigGo Finance</t>
-        </is>
-      </c>
-      <c r="C15" s="20" t="inlineStr">
-        <is>
-          <t>https://finance.biggo.com/news/KR_000660.KS_2026-07-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="n">
-        <v>13</v>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Chip stocks shed $1tn in selloff — CNBC</t>
-        </is>
-      </c>
-      <c r="C16" s="20" t="inlineStr">
-        <is>
-          <t>https://www.cnbc.com/2026/07/29/chip-selloff-sk-hynix-samsung-softbank.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="n">
-        <v>14</v>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Asian tech stocks drop, SK Hynix -10% — CNBC</t>
-        </is>
-      </c>
-      <c r="C17" s="20" t="inlineStr">
-        <is>
-          <t>https://www.cnbc.com/2026/08/06/asia-tech-selloff-wall-street-samsung-sk-hynix.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="9" t="n">
-        <v>15</v>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Emergency meeting as W864tn leaves market — Yahoo Finance</t>
-        </is>
-      </c>
-      <c r="C18" s="20" t="inlineStr">
-        <is>
-          <t>https://finance.yahoo.com/markets/world-indices/articles/south-korea-holds-emergency-meeting-103240901.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="n">
-        <v>16</v>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>Kospi rout puts Lee government on alert — Bloomingbit</t>
-        </is>
-      </c>
-      <c r="C19" s="20" t="inlineStr">
-        <is>
-          <t>https://en.bloomingbit.io/feed/news/117526</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="9" t="n">
-        <v>17</v>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>NPS: an amplifier, not a stabilizer — Korea JoongAng Daily</t>
-        </is>
-      </c>
-      <c r="C20" s="20" t="inlineStr">
-        <is>
-          <t>https://www.koreajoongangdaily.com/opinion/nps-becomes-an-amplifier-not-a-stabilizer/12782277</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="n">
-        <v>18</v>
-      </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>KOSPI falls to 6,200 level, 6 August — Seoul Economic Daily</t>
-        </is>
-      </c>
-      <c r="C21" s="20" t="inlineStr">
-        <is>
-          <t>https://en.sedaily.com/finance/2026/08/06/kospi-falls-to-6200-level-as-chip-giants-plunge-kosdaq</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="n">
-        <v>19</v>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>Hyperscalers plan $725bn 2026 AI capex — AI Weekly</t>
-        </is>
-      </c>
-      <c r="C22" s="20" t="inlineStr">
-        <is>
-          <t>https://aiweekly.co/alerts/amazon-microsoft-alphabet-meta-plan-725b-ai-capex-in-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Michael Burry warns of 1987-type fall — CNBC</t>
-        </is>
-      </c>
-      <c r="C23" s="20" t="inlineStr">
-        <is>
-          <t>https://www.cnbc.com/2026/08/04/michael-burry-bets-against-rally-we-are-near-a-major-top.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="9" t="n">
-        <v>21</v>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>J.P. Morgan: AI investment cycle not derailed — CNBC</t>
-        </is>
-      </c>
-      <c r="C24" s="20" t="inlineStr">
-        <is>
-          <t>https://www.cnbc.com/2026/08/06/asia-tech-sell-off-has-not-derailed-ai-investment-cycle-jp-morgan-says.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>SKHY / MU daily price data — Twelve Data API</t>
-        </is>
-      </c>
-      <c r="C25" s="20" t="inlineStr">
-        <is>
-          <t>https://twelvedata.com (live-fetched 2026-08-07, see Price Data sheet)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="9" t="n">
-        <v>23</v>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>KOSPI's record +17.91% single-day gain, 31 July — TradingKey</t>
-        </is>
-      </c>
-      <c r="C26" s="20" t="inlineStr">
-        <is>
-          <t>https://www.tradingkey.com/analysis/stocks/us-stocks/262067341-kospi-surged-17-9-percent-largest-single-day-gain-history-july-31-2026-tradingkey</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="n">
-        <v>24</v>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>SanDisk/Western Digital guidance miss drags SK Hynix, Micron — TradingKey</t>
-        </is>
-      </c>
-      <c r="C27" s="20" t="inlineStr">
-        <is>
-          <t>https://www.tradingkey.com/analysis/stocks/us-stocks/262082159-us-stock-sndk-wdc-skhy-mu-ai-tradingkey</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="9" t="n">
-        <v>25</v>
-      </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>KOSPI all-time high of 9,385.59 on 19 June — IndMoney</t>
-        </is>
-      </c>
-      <c r="C28" s="20" t="inlineStr">
-        <is>
-          <t>https://www.indmoney.com/blog/us-stocks/kospi-index-crash-analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="n">
-        <v>26</v>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>KOSPI slides over 4% as tech shares tumble, 6 August — Korea JoongAng Daily</t>
-        </is>
-      </c>
-      <c r="C29" s="20" t="inlineStr">
-        <is>
-          <t>https://www.koreajoongangdaily.com/business/kospi-slides-over-4-as-tech-shares-take-a-tumble/12812355</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId26"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix chart index base to day one, justify the MU comparison and window start
Index was set to 7/14 (the crash date) instead of the first trading day,
which is non-standard and needed justifying. Switched both the site chart
and the workbook's Indexed columns to index off 7/10 (SKHY's actual Nasdaq
debut - there's no earlier data for this security to show). Kept 7/14 as
the reference date for the peak-to-trough drawdown stat specifically, since
that's the real event date the story hinges on, and added a robustness
check showing the conclusion doesn't change if MU's own true high (23 July)
is used instead. Also restored the chart, which had been stripped from the
xlsx by a manual edit outside of this script, and made the "why compare to
Micron" and "why does the data start 7/10" reasoning explicit in both the
article text and the workbook.
</commit_message>
<xml_diff>
--- a/public/downloads/korea-leverage-crash-data.xlsx
+++ b/public/downloads/korea-leverage-crash-data.xlsx
@@ -251,7 +251,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>SKHY (SK Hynix ADR) vs. MU (Micron), indexed to 100 on 2026-07-14</a:t>
+              <a:t>SKHY (SK Hynix ADR) vs. MU (Micron), indexed to 100 on 2026-07-10 (SKHY's first trading day)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -379,7 +379,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Indexed (7/14 = 100)</a:t>
+                  <a:t>Indexed (7/10 = 100)</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>SKHY Indexed (7/14=100)</t>
+          <t>SKHY Indexed (7/10=100)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>MU Indexed (7/14=100)</t>
+          <t>MU Indexed (7/10=100)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -1062,7 +1062,7 @@
         <v>168.01</v>
       </c>
       <c r="C4" s="6">
-        <f>B4/$B$6*100</f>
+        <f>B4/$B$4*100</f>
         <v/>
       </c>
       <c r="D4" s="7" t="n"/>
@@ -1070,7 +1070,7 @@
         <v>979.3</v>
       </c>
       <c r="F4" s="6">
-        <f>E4/$E$6*100</f>
+        <f>E4/$E$4*100</f>
         <v/>
       </c>
       <c r="G4" s="7" t="n"/>
@@ -1085,7 +1085,7 @@
         <v>152.35</v>
       </c>
       <c r="C5" s="6">
-        <f>B5/$B$6*100</f>
+        <f>B5/$B$4*100</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -1096,7 +1096,7 @@
         <v>937</v>
       </c>
       <c r="F5" s="6">
-        <f>E5/$E$6*100</f>
+        <f>E5/$E$4*100</f>
         <v/>
       </c>
       <c r="G5" s="8">
@@ -1114,7 +1114,7 @@
         <v>193.92</v>
       </c>
       <c r="C6" s="6">
-        <f>B6/$B$6*100</f>
+        <f>B6/$B$4*100</f>
         <v/>
       </c>
       <c r="D6" s="8">
@@ -1125,7 +1125,7 @@
         <v>983.12</v>
       </c>
       <c r="F6" s="6">
-        <f>E6/$E$6*100</f>
+        <f>E6/$E$4*100</f>
         <v/>
       </c>
       <c r="G6" s="8">
@@ -1143,7 +1143,7 @@
         <v>176.46</v>
       </c>
       <c r="C7" s="6">
-        <f>B7/$B$6*100</f>
+        <f>B7/$B$4*100</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -1154,7 +1154,7 @@
         <v>904.28</v>
       </c>
       <c r="F7" s="6">
-        <f>E7/$E$6*100</f>
+        <f>E7/$E$4*100</f>
         <v/>
       </c>
       <c r="G7" s="8">
@@ -1172,7 +1172,7 @@
         <v>152.31</v>
       </c>
       <c r="C8" s="6">
-        <f>B8/$B$6*100</f>
+        <f>B8/$B$4*100</f>
         <v/>
       </c>
       <c r="D8" s="8">
@@ -1183,7 +1183,7 @@
         <v>853.2</v>
       </c>
       <c r="F8" s="6">
-        <f>E8/$E$6*100</f>
+        <f>E8/$E$4*100</f>
         <v/>
       </c>
       <c r="G8" s="8">
@@ -1201,7 +1201,7 @@
         <v>154.03</v>
       </c>
       <c r="C9" s="6">
-        <f>B9/$B$6*100</f>
+        <f>B9/$B$4*100</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -1212,7 +1212,7 @@
         <v>848.95</v>
       </c>
       <c r="F9" s="6">
-        <f>E9/$E$6*100</f>
+        <f>E9/$E$4*100</f>
         <v/>
       </c>
       <c r="G9" s="8">
@@ -1230,7 +1230,7 @@
         <v>151.16</v>
       </c>
       <c r="C10" s="6">
-        <f>B10/$B$6*100</f>
+        <f>B10/$B$4*100</f>
         <v/>
       </c>
       <c r="D10" s="8">
@@ -1241,7 +1241,7 @@
         <v>865.46</v>
       </c>
       <c r="F10" s="6">
-        <f>E10/$E$6*100</f>
+        <f>E10/$E$4*100</f>
         <v/>
       </c>
       <c r="G10" s="8">
@@ -1259,7 +1259,7 @@
         <v>171.94</v>
       </c>
       <c r="C11" s="6">
-        <f>B11/$B$6*100</f>
+        <f>B11/$B$4*100</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -1270,7 +1270,7 @@
         <v>970.8200000000001</v>
       </c>
       <c r="F11" s="6">
-        <f>E11/$E$6*100</f>
+        <f>E11/$E$4*100</f>
         <v/>
       </c>
       <c r="G11" s="8">
@@ -1288,7 +1288,7 @@
         <v>165.27</v>
       </c>
       <c r="C12" s="6">
-        <f>B12/$B$6*100</f>
+        <f>B12/$B$4*100</f>
         <v/>
       </c>
       <c r="D12" s="8">
@@ -1299,7 +1299,7 @@
         <v>959.48</v>
       </c>
       <c r="F12" s="6">
-        <f>E12/$E$6*100</f>
+        <f>E12/$E$4*100</f>
         <v/>
       </c>
       <c r="G12" s="8">
@@ -1317,7 +1317,7 @@
         <v>169.5</v>
       </c>
       <c r="C13" s="6">
-        <f>B13/$B$6*100</f>
+        <f>B13/$B$4*100</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -1328,7 +1328,7 @@
         <v>990.21</v>
       </c>
       <c r="F13" s="6">
-        <f>E13/$E$6*100</f>
+        <f>E13/$E$4*100</f>
         <v/>
       </c>
       <c r="G13" s="8">
@@ -1346,7 +1346,7 @@
         <v>154.57</v>
       </c>
       <c r="C14" s="6">
-        <f>B14/$B$6*100</f>
+        <f>B14/$B$4*100</f>
         <v/>
       </c>
       <c r="D14" s="8">
@@ -1357,7 +1357,7 @@
         <v>920.95</v>
       </c>
       <c r="F14" s="6">
-        <f>E14/$E$6*100</f>
+        <f>E14/$E$4*100</f>
         <v/>
       </c>
       <c r="G14" s="8">
@@ -1375,7 +1375,7 @@
         <v>143.02</v>
       </c>
       <c r="C15" s="6">
-        <f>B15/$B$6*100</f>
+        <f>B15/$B$4*100</f>
         <v/>
       </c>
       <c r="D15" s="8">
@@ -1386,7 +1386,7 @@
         <v>900.2</v>
       </c>
       <c r="F15" s="6">
-        <f>E15/$E$6*100</f>
+        <f>E15/$E$4*100</f>
         <v/>
       </c>
       <c r="G15" s="8">
@@ -1404,7 +1404,7 @@
         <v>130.17</v>
       </c>
       <c r="C16" s="6">
-        <f>B16/$B$6*100</f>
+        <f>B16/$B$4*100</f>
         <v/>
       </c>
       <c r="D16" s="8">
@@ -1415,7 +1415,7 @@
         <v>820.53</v>
       </c>
       <c r="F16" s="6">
-        <f>E16/$E$6*100</f>
+        <f>E16/$E$4*100</f>
         <v/>
       </c>
       <c r="G16" s="8">
@@ -1433,7 +1433,7 @@
         <v>126.79</v>
       </c>
       <c r="C17" s="6">
-        <f>B17/$B$6*100</f>
+        <f>B17/$B$4*100</f>
         <v/>
       </c>
       <c r="D17" s="8">
@@ -1444,7 +1444,7 @@
         <v>739</v>
       </c>
       <c r="F17" s="6">
-        <f>E17/$E$6*100</f>
+        <f>E17/$E$4*100</f>
         <v/>
       </c>
       <c r="G17" s="8">
@@ -1462,7 +1462,7 @@
         <v>149</v>
       </c>
       <c r="C18" s="6">
-        <f>B18/$B$6*100</f>
+        <f>B18/$B$4*100</f>
         <v/>
       </c>
       <c r="D18" s="8">
@@ -1473,7 +1473,7 @@
         <v>874.66</v>
       </c>
       <c r="F18" s="6">
-        <f>E18/$E$6*100</f>
+        <f>E18/$E$4*100</f>
         <v/>
       </c>
       <c r="G18" s="8">
@@ -1491,7 +1491,7 @@
         <v>143.73</v>
       </c>
       <c r="C19" s="6">
-        <f>B19/$B$6*100</f>
+        <f>B19/$B$4*100</f>
         <v/>
       </c>
       <c r="D19" s="8">
@@ -1502,7 +1502,7 @@
         <v>823.03</v>
       </c>
       <c r="F19" s="6">
-        <f>E19/$E$6*100</f>
+        <f>E19/$E$4*100</f>
         <v/>
       </c>
       <c r="G19" s="8">
@@ -1520,7 +1520,7 @@
         <v>142.72</v>
       </c>
       <c r="C20" s="6">
-        <f>B20/$B$6*100</f>
+        <f>B20/$B$4*100</f>
         <v/>
       </c>
       <c r="D20" s="8">
@@ -1531,7 +1531,7 @@
         <v>829.5</v>
       </c>
       <c r="F20" s="6">
-        <f>E20/$E$6*100</f>
+        <f>E20/$E$4*100</f>
         <v/>
       </c>
       <c r="G20" s="8">
@@ -1549,7 +1549,7 @@
         <v>154.38</v>
       </c>
       <c r="C21" s="6">
-        <f>B21/$B$6*100</f>
+        <f>B21/$B$4*100</f>
         <v/>
       </c>
       <c r="D21" s="8">
@@ -1560,7 +1560,7 @@
         <v>892.67</v>
       </c>
       <c r="F21" s="6">
-        <f>E21/$E$6*100</f>
+        <f>E21/$E$4*100</f>
         <v/>
       </c>
       <c r="G21" s="8">
@@ -1578,7 +1578,7 @@
         <v>151.03</v>
       </c>
       <c r="C22" s="6">
-        <f>B22/$B$6*100</f>
+        <f>B22/$B$4*100</f>
         <v/>
       </c>
       <c r="D22" s="8">
@@ -1589,7 +1589,7 @@
         <v>893.1900000000001</v>
       </c>
       <c r="F22" s="6">
-        <f>E22/$E$6*100</f>
+        <f>E22/$E$4*100</f>
         <v/>
       </c>
       <c r="G22" s="8">
@@ -1607,7 +1607,7 @@
         <v>145.87</v>
       </c>
       <c r="C23" s="6">
-        <f>B23/$B$6*100</f>
+        <f>B23/$B$4*100</f>
         <v/>
       </c>
       <c r="D23" s="8">
@@ -1618,7 +1618,7 @@
         <v>898.97</v>
       </c>
       <c r="F23" s="6">
-        <f>E23/$E$6*100</f>
+        <f>E23/$E$4*100</f>
         <v/>
       </c>
       <c r="G23" s="8">
@@ -1629,21 +1629,21 @@
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>Why MU, and why this matters for the thesis</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="105" customHeight="1">
+          <t>Why this window, why MU, and why this matters for the thesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="135" customHeight="1">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>MU (Micron) is the control group. It's a comparable, US-listed memory-chip maker riding the exact same global AI/memory demand cycle as SK Hynix — but with zero exposure to Korea's leveraged-ETF machinery, margin calls, or forced retail liquidations, because it isn't a Korean stock. If Korea-specific leverage were the main driver of SK Hynix's crash, MU should have barely moved over the same window. It didn't: MU fell 24.8% while SKHY fell 34.6% — nearly as much, on a stock with none of Korea's leverage mechanics attached to it. That's the evidence for the article's central claim: most of SK Hynix's drawdown is the same global correction that hit an unlevered peer almost as hard. Korea's leverage machinery accounts for the incremental ~10 points below (see 'Implied Korea-specific incremental damage') and for nearly all of the margin-call/social fallout — not for the bulk of the price move itself.</t>
+          <t>The window starts 10 July because that's SKHY's actual first trading day — SK Hynix's Nasdaq ADR listed that morning, so there is no earlier price history for this specific security to show; the index (column C) is set to 100 there, on day one, the normal convention, not on some later date chosen to flatter the result. MU (Micron) is the control group: a comparable, US-listed memory-chip maker riding the same global AI/memory demand cycle as SK Hynix, but with zero exposure to Korea's leveraged-ETF machinery, margin calls, or forced retail liquidations, because it isn't a Korean stock. If Korea-specific leverage were the main driver of SK Hynix's crash, MU should have barely moved over the same window. It didn't. The peak-to-trough stat below uses 14 July as the reference date for BOTH stocks — not because it's literally MU's own peak (MU actually closed slightly higher, at $990.21, on 23 July) but because 14 July is the real event date this whole story hinges on (Seoul -15%, the ADR +27%, same day). As a check: measured from MU's own true high on 23 July instead, its decline to the 29 July trough is -25.4% — barely different from the -24.8% below. The conclusion doesn't depend on which exact date you pick.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Peak (7/14) to trough (7/29):</t>
+          <t>Same-window decline, 14 Jul to 29 Jul (see note above):</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Fix the Excel chart's missing axis labels and improve legibility
Found three real bugs causing WPS/Excel to render the chart with no y-axis
numbers and no x-axis dates: openpyxl leaves axis delete/tickLblPos as None
(some viewers treat that as hidden rather than the spec default of visible),
it defaults BOTH axes' axPos to "l" (left) instead of putting the category
axis at the bottom, and set_categories() always wraps the reference in a
NumRef even when the underlying cells are text - so a text-based date axis
had no valid reference type at all. Fixed all three explicitly. Also
shortened the date column to "Jul 10" style for a readable x-axis, thickened
the lines, enlarged the chart, and added a caption pointing at the actual
divergence the chart is meant to show.
</commit_message>
<xml_diff>
--- a/public/downloads/korea-leverage-crash-data.xlsx
+++ b/public/downloads/korea-leverage-crash-data.xlsx
@@ -269,7 +269,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln w="22000">
               <a:solidFill>
                 <a:srgbClr val="BC5B33"/>
               </a:solidFill>
@@ -278,7 +278,7 @@
           </spPr>
           <marker>
             <symbol val="circle"/>
-            <size val="4"/>
+            <size val="5"/>
             <spPr>
               <a:ln>
                 <a:prstDash val="solid"/>
@@ -286,9 +286,9 @@
             </spPr>
           </marker>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Price Data'!$A$4:$A$23</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -306,7 +306,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln w="22000">
               <a:solidFill>
                 <a:srgbClr val="2F6F9F"/>
               </a:solidFill>
@@ -315,7 +315,7 @@
           </spPr>
           <marker>
             <symbol val="circle"/>
-            <size val="4"/>
+            <size val="5"/>
             <spPr>
               <a:ln>
                 <a:prstDash val="solid"/>
@@ -323,9 +323,9 @@
             </spPr>
           </marker>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Price Data'!$A$4:$A$23</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -342,7 +342,8 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <delete val="0"/>
+        <axPos val="b"/>
         <title>
           <tx>
             <rich>
@@ -358,16 +359,19 @@
             </rich>
           </tx>
         </title>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="low"/>
         <crossAx val="100"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="2"/>
       </catAx>
       <valAx>
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -385,8 +389,10 @@
             </rich>
           </tx>
         </title>
-        <majorTickMark val="none"/>
+        <numFmt formatCode="0" sourceLinked="0"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
@@ -408,7 +414,7 @@
       <row>32</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8640000" cy="3240000"/>
+    <ext cx="10080000" cy="3960000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -996,7 +1002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1055,7 +1061,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>Jul 10</t>
         </is>
       </c>
       <c r="B4" s="5" t="n">
@@ -1078,7 +1084,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>Jul 13</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
@@ -1107,7 +1113,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>Jul 14</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
@@ -1136,7 +1142,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>Jul 15</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
@@ -1165,7 +1171,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>Jul 16</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
@@ -1194,7 +1200,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>Jul 17</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
@@ -1223,7 +1229,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>Jul 20</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
@@ -1252,7 +1258,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>Jul 21</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
@@ -1281,7 +1287,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>Jul 22</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
@@ -1310,7 +1316,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>Jul 23</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
@@ -1339,7 +1345,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>Jul 24</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
@@ -1368,7 +1374,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>Jul 27</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
@@ -1397,7 +1403,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>Jul 28</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
@@ -1426,7 +1432,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>Jul 29</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
@@ -1455,7 +1461,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>Jul 30</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
@@ -1484,7 +1490,7 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>Jul 31</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
@@ -1513,7 +1519,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>Aug 3</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
@@ -1542,7 +1548,7 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>Aug 4</t>
         </is>
       </c>
       <c r="B21" s="5" t="n">
@@ -1571,7 +1577,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>Aug 5</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
@@ -1600,7 +1606,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>Aug 6</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
@@ -1678,57 +1684,57 @@
         <v/>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="26" customHeight="1">
       <c r="A32" s="12" t="inlineStr">
         <is>
-          <t>Chart follows the Timeline sheet's dates — see annotations there for what each move corresponds to.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="9" t="inlineStr">
+          <t>Watch the gap between the two lines from 14 Jul onward — before that they move together; the gap that opens up after is the Korea-specific piece of this story. Chart follows the Timeline sheet's dates — see annotations there for what each move corresponds to.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="inlineStr">
         <is>
           <t>Sources for the price data on this sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="13" t="inlineStr">
-        <is>
-          <t>- SKHY and MU daily OHLCV — Twelve Data API (twelvedata.com), live-fetched 2026-08-07. Not a live feed: a dated snapshot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="13" t="inlineStr">
-        <is>
-          <t>- SK Hynix Seoul-listed shares -15.37% on 7/14 — Advisor Perspectives, https://www.advisorperspectives.com/articles/2026/07/13/sk-hynix-shares-plunge-record-deepening-korea-selloff</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="13" t="inlineStr">
-        <is>
-          <t>- KOSPI record +17.91% single-day gain, 7/31 — TradingKey, https://www.tradingkey.com/analysis/stocks/us-stocks/262067341-kospi-surged-17-9-percent-largest-single-day-gain-history-july-31-2026-tradingkey</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="13" t="inlineStr">
-        <is>
-          <t>- KOSPI all-time high 9,385.59 on 6/19 — IndMoney, https://www.indmoney.com/blog/us-stocks/kospi-index-crash-analysis</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="13" t="inlineStr">
         <is>
-          <t>- SanDisk/Western Digital guidance miss driving the 8/6 selloff — TradingKey, https://www.tradingkey.com/analysis/stocks/us-stocks/262082159-us-stock-sndk-wdc-skhy-mu-ai-tradingkey</t>
+          <t>- SKHY and MU daily OHLCV — Twelve Data API (twelvedata.com), live-fetched 2026-08-07. Not a live feed: a dated snapshot.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>- SK Hynix Seoul-listed shares -15.37% on 7/14 — Advisor Perspectives, https://www.advisorperspectives.com/articles/2026/07/13/sk-hynix-shares-plunge-record-deepening-korea-selloff</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="13" t="inlineStr">
+        <is>
+          <t>- KOSPI record +17.91% single-day gain, 7/31 — TradingKey, https://www.tradingkey.com/analysis/stocks/us-stocks/262067341-kospi-surged-17-9-percent-largest-single-day-gain-history-july-31-2026-tradingkey</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="13" t="inlineStr">
+        <is>
+          <t>- KOSPI all-time high 9,385.59 on 6/19 — IndMoney, https://www.indmoney.com/blog/us-stocks/kospi-index-crash-analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="13" t="inlineStr">
+        <is>
+          <t>- SanDisk/Western Digital guidance miss driving the 8/6 selloff — TradingKey, https://www.tradingkey.com/analysis/stocks/us-stocks/262082159-us-stock-sndk-wdc-skhy-mu-ai-tradingkey</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="13" t="inlineStr">
         <is>
           <t>- Samsung -6.3% close, SK Hynix selloff, 8/6 — Korea JoongAng Daily, https://www.koreajoongangdaily.com/business/kospi-slides-over-4-as-tech-shares-take-a-tumble/12812355</t>
         </is>

</xml_diff>

<commit_message>
Rewrite around the corrected finding: the ADR's own drawdown matches Micron's
Reordered the two sections so the ADR/Seoul split (why 7/14 was an inflated
reference point) comes before the comparison, then rebuilt the comparison
itself around the honest, day-1-indexed numbers: SKHY -24.53% vs MU -24.54%
to the 29 July trough, essentially identical, instead of the old 34.6%/24.8%
framing that only existed because it measured from SKHY's own IPO-week pop.
Framed explicitly around headlines reaching for the biggest defensible
number rather than the most accurate one - not an accusation that any
source got facts wrong, just that the "35% crash" doesn't survive checking
against an honest starting point. Updated the tagline, intro, chart note/
annotations, and "My view" to match. Excel workbook's Price Data sheet now
leads with the honest day-1 comparison and shows the headline-style 14 Jul
number only as a labeled secondary reference.
</commit_message>
<xml_diff>
--- a/public/downloads/korea-leverage-crash-data.xlsx
+++ b/public/downloads/korea-leverage-crash-data.xlsx
@@ -124,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -145,6 +145,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -411,7 +412,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>32</row>
+      <row>36</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10080000" cy="3960000"/>
@@ -1002,7 +1003,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1635,21 +1636,21 @@
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>Why this window, why MU, and why this matters for the thesis</t>
+          <t>Why this window, why MU, and the number headlines actually reported</t>
         </is>
       </c>
     </row>
     <row r="26" ht="135" customHeight="1">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>The window starts 10 July because that's SKHY's actual first trading day — SK Hynix's Nasdaq ADR listed that morning, so there is no earlier price history for this specific security to show; the index (column C) is set to 100 there, on day one, the normal convention, not on some later date chosen to flatter the result. MU (Micron) is the control group: a comparable, US-listed memory-chip maker riding the same global AI/memory demand cycle as SK Hynix, but with zero exposure to Korea's leveraged-ETF machinery, margin calls, or forced retail liquidations, because it isn't a Korean stock. If Korea-specific leverage were the main driver of SK Hynix's crash, MU should have barely moved over the same window. It didn't. The peak-to-trough stat below uses 14 July as the reference date for BOTH stocks — not because it's literally MU's own peak (MU actually closed slightly higher, at $990.21, on 23 July) but because 14 July is the real event date this whole story hinges on (Seoul -15%, the ADR +27%, same day). As a check: measured from MU's own true high on 23 July instead, its decline to the 29 July trough is -25.4% — barely different from the -24.8% below. The conclusion doesn't depend on which exact date you pick.</t>
+          <t>Every article on this crash cites a large SK Hynix drawdown — not fabricated, but measured from 14 July, SKHY's own post-IPO peak (it had popped 27% in two days on first-week ADR demand, unrelated to Korea's crash). That's the biggest defensible number, not the most accurate one. The window here starts 10 July instead — SKHY's actual first trading day, the normal 'index to day one' convention, not a later date chosen to flatter the result. MU (Micron) is the control group: a comparable, US-listed memory-chip maker on the same global AI/memory demand cycle, with zero exposure to Korea's leveraged-ETF machinery, margin calls, or forced liquidations, because it isn't a Korean stock. Measured honestly (see 'the honest comparison' below), SKHY and MU fell by statistically the same amount to the 29 July trough — meaning almost none of the ADR's own price decline was actually Korea-specific. The 'headline' 14-Jul-to-trough numbers are shown too, for reference, but that gap is mostly SKHY's own IPO-week pop unwinding, not incremental Korea-leverage damage.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Same-window decline, 14 Jul to 29 Jul (see note above):</t>
+          <t>Day 1 (10 Jul) to trough (29 Jul) — the honest comparison:</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
@@ -1658,7 +1659,7 @@
         </is>
       </c>
       <c r="C28" s="11">
-        <f>B17/B6-1</f>
+        <f>B17/B4-1</f>
         <v/>
       </c>
     </row>
@@ -1669,14 +1670,14 @@
         </is>
       </c>
       <c r="C29" s="11">
-        <f>E17/E6-1</f>
+        <f>E17/E4-1</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Implied 'Korea-specific' incremental damage</t>
+          <t>Gap — should be ~0 if this were really a Korea-specific price story</t>
         </is>
       </c>
       <c r="C30" s="11">
@@ -1684,57 +1685,95 @@
         <v/>
       </c>
     </row>
-    <row r="32" ht="26" customHeight="1">
-      <c r="A32" s="12" t="inlineStr">
-        <is>
-          <t>Watch the gap between the two lines from 14 Jul onward — before that they move together; the gap that opens up after is the Korea-specific piece of this story. Chart follows the Timeline sheet's dates — see annotations there for what each move corresponds to.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="9" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>For reference — 14 Jul (the date headlines use) to trough:</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>SKHY drawdown</t>
+        </is>
+      </c>
+      <c r="C32" s="12">
+        <f>B17/B6-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>MU drawdown (same reference date)</t>
+        </is>
+      </c>
+      <c r="C33" s="12">
+        <f>E17/E6-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Gap — mostly SKHY's own IPO-week pop, not incremental Korea damage</t>
+        </is>
+      </c>
+      <c r="C34" s="12">
+        <f>C32-C33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="26" customHeight="1">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>Watch where the lines land, not just where they spread: SKHY spikes on 14 Jul (its own IPO-week pop), but by the 29 Jul trough both lines are back on top of each other. That convergence, not the 14 Jul gap, is the actual finding. Chart follows the Timeline sheet's dates — see annotations there for what each move corresponds to.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="9" t="inlineStr">
         <is>
           <t>Sources for the price data on this sheet</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="13" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="14" t="inlineStr">
         <is>
           <t>- SKHY and MU daily OHLCV — Twelve Data API (twelvedata.com), live-fetched 2026-08-07. Not a live feed: a dated snapshot.</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="13" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="14" t="inlineStr">
         <is>
           <t>- SK Hynix Seoul-listed shares -15.37% on 7/14 — Advisor Perspectives, https://www.advisorperspectives.com/articles/2026/07/13/sk-hynix-shares-plunge-record-deepening-korea-selloff</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="13" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="14" t="inlineStr">
         <is>
           <t>- KOSPI record +17.91% single-day gain, 7/31 — TradingKey, https://www.tradingkey.com/analysis/stocks/us-stocks/262067341-kospi-surged-17-9-percent-largest-single-day-gain-history-july-31-2026-tradingkey</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="13" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="14" t="inlineStr">
         <is>
           <t>- KOSPI all-time high 9,385.59 on 6/19 — IndMoney, https://www.indmoney.com/blog/us-stocks/kospi-index-crash-analysis</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="13" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="14" t="inlineStr">
         <is>
           <t>- SanDisk/Western Digital guidance miss driving the 8/6 selloff — TradingKey, https://www.tradingkey.com/analysis/stocks/us-stocks/262082159-us-stock-sndk-wdc-skhy-mu-ai-tradingkey</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="13" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="14" t="inlineStr">
         <is>
           <t>- Samsung -6.3% close, SK Hynix selloff, 8/6 — Korea JoongAng Daily, https://www.koreajoongangdaily.com/business/kospi-slides-over-4-as-tech-shares-take-a-tumble/12812355</t>
         </is>
@@ -1793,12 +1832,12 @@
           <t>Single-stock leveraged ETFs launched</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>27 May 2026</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>2x daily return products tied to Samsung / SK Hynix</t>
         </is>
@@ -1810,12 +1849,12 @@
           <t>Net retail purchases of leveraged ETFs</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>~W14tn (~$9.4bn)</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>vs. ~W2tn from foreign investors</t>
         </is>
@@ -1827,12 +1866,12 @@
           <t>Peak outstanding leveraged bets</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>W29.2tn (~$19.7bn)</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="16" t="inlineStr">
         <is>
           <t>Early July 2026</t>
         </is>
@@ -1844,12 +1883,12 @@
           <t>Retail accounts hitting margin calls</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>1,200,000+</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>As of 13 July 2026</t>
         </is>
@@ -1861,12 +1900,12 @@
           <t>Accounts forcibly liquidated</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>320,000 - 360,000</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>As of mid-July 2026</t>
         </is>
@@ -1878,12 +1917,12 @@
           <t>Total forced liquidation value</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>W2.3tn</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>Over ~2.5 months</t>
         </is>
@@ -1895,12 +1934,12 @@
           <t>New minimum deposit for leveraged investors (post-crisis)</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>W30m (~$20,000)</t>
         </is>
       </c>
-      <c r="C10" s="15" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>Tripled by the FSC, late July 2026</t>
         </is>
@@ -1912,12 +1951,12 @@
           <t>KOSPI single 2-day value wipeout</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>W864.5tn</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="C11" s="16" t="inlineStr">
         <is>
           <t>Triggered the 29 July emergency government meeting</t>
         </is>
@@ -1929,12 +1968,12 @@
           <t>President Lee Jae-myung disapproval rating</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>&gt;50%</t>
         </is>
       </c>
-      <c r="C12" s="15" t="inlineStr">
+      <c r="C12" s="16" t="inlineStr">
         <is>
           <t>First time in his term, per BigGo Finance / Bloombit reporting</t>
         </is>
@@ -1984,85 +2023,85 @@
       </c>
     </row>
     <row r="4" ht="70" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>SK Hynix Q2 result</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Revenue W79.32tn, +257% YoY, 76% operating margin — a genuine record quarter. 'Miss' vs. consensus (~W84tn) was a shipment-timing issue (HBM4 recognition slipping to Q3), not a demand problem.</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>Even a record quarter missed elevated Street expectations — a real sign the market had priced in near-perfection, leaving no room for anything less.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="70" customHeight="1">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Underlying AI demand</t>
         </is>
       </c>
-      <c r="B5" s="17" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>Hyperscaler 2026 capex guidance: Amazon $200bn, Alphabet $175-185bn, Meta $115-135bn, Microsoft $190bn — $725bn combined, +77% YoY. Evercore/BofA model &gt;$1tn combined for 2027. S&amp;P Global's July PMI showed the fastest tech-equipment output growth since May 2021.</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>Crowding and leverage across the whole AI trade (not just Korea) means positioning, not fundamentals, is doing a lot of the work in the price — a similar unwind could happen anywhere sentiment cracks next.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="70" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Analyst / investor commentary</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>J.P. Morgan (6 Aug note): the sell-off 'had not derailed' the AI investment cycle; 'we do not see any fundamental indicators that signal meaningful weakness in the next 6-12 months.'</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="C6" s="19" t="inlineStr">
         <is>
           <t>Michael Burry (4 Aug Substack): 'I continue to believe it is possible we are near a major top, and possibly a 1987-type fall.'</t>
         </is>
       </c>
     </row>
     <row r="7" ht="70" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>China competitive threat</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Currently immaterial in scale: ~5 domestic DUV units expected in 2026 vs. ASML's ~130 immersion systems; China's tools reportedly still lag ASML's technology.</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
+      <c r="C7" s="19" t="inlineStr">
         <is>
           <t>A real, credible first step toward Chinese self-sufficiency in a category it has never mass-produced before — a genuine multi-year strategic risk even if not a 2026-2027 supply/demand issue.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="70" customHeight="1">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>2027-2028 capacity</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>New capacity gives SK Hynix/Samsung/Micron room to keep growing into real, still-accelerating demand.</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
+      <c r="C8" s="19" t="inlineStr">
         <is>
           <t>Samsung, SK Hynix, Micron and Kioxia are all adding capacity simultaneously, due to reach volume in late 2027/2028 — right as hyperscaler capex growth may naturally decelerate off this year's exceptional base. The same setup that has ended every prior memory cycle.</t>
         </is>

</xml_diff>